<commit_message>
Transferring project to new account
</commit_message>
<xml_diff>
--- a/Emp_data.xlsx
+++ b/Emp_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,72 +417,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>emp_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>emp_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>emp_team</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Total_leaves</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Half_Day</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Leaves</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Remaining_Leaves</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>is_admin</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>WFH_count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Contract_Type</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Contract_Start_Date</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Contract_End_Date</t>
         </is>
@@ -518,22 +506,22 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>10.5</v>
+        <v>14</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -565,13 +553,13 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -609,13 +597,13 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -653,13 +641,13 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -694,16 +682,16 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -741,13 +729,13 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -782,22 +770,22 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>4.5</v>
+        <v>14</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -829,13 +817,13 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -873,13 +861,13 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -917,13 +905,13 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -964,7 +952,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>14</v>
@@ -1002,16 +990,16 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix: include all missing changes in attendance_manager and other files
</commit_message>
<xml_diff>
--- a/Emp_data.xlsx
+++ b/Emp_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,26 @@
           <t>is_manager</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Leaves_This_Year</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Leaves_Carried_Forward</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Contract_Year_Start</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -511,7 +531,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
@@ -520,13 +540,13 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -534,11 +554,23 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
         <v>0</v>
       </c>
+      <c r="P2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -546,7 +578,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ismail Anwer</t>
+          <t>Ismail Anwar</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -581,11 +613,23 @@
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
         <v>0</v>
       </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -593,7 +637,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Haris saeed</t>
+          <t>Haris Saeed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -628,11 +672,23 @@
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2025-06-15</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
         <v>0</v>
       </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -675,11 +731,23 @@
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
         <v>0</v>
       </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -722,11 +790,27 @@
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2025-02-20</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
         <v>1</v>
       </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>03365111740</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -769,11 +853,23 @@
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2025-04-10</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
         <v>0</v>
       </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -808,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -816,11 +912,23 @@
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
         <v>0</v>
       </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -863,11 +971,23 @@
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2025-11-15</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="n">
         <v>0</v>
       </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -875,7 +995,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sajeel Faseehi</t>
+          <t>Sajeel Fasihi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -899,7 +1019,7 @@
         <v>14</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -910,10 +1030,26 @@
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>03245494440</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -927,7 +1063,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Poppi</t>
+          <t>LHM</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -957,11 +1093,23 @@
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="n">
         <v>0</v>
       </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -969,7 +1117,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hatif</t>
+          <t>Hatif Javed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1004,11 +1152,27 @@
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="n">
         <v>1</v>
       </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>03365404410</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1016,7 +1180,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Moeed</t>
+          <t>Moeed Iftikhar</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1051,11 +1215,23 @@
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
         <v>0</v>
       </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1098,11 +1274,23 @@
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2025-01-25</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
         <v>0</v>
       </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1110,12 +1298,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Atti ullah</t>
+          <t>Attiullah</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Internee</t>
+          <t>Overstock</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1145,11 +1333,23 @@
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2025-03-30</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
         <v>0</v>
       </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1192,11 +1392,23 @@
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
         <v>0</v>
       </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1204,7 +1416,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jhanzaib</t>
+          <t>Jahanzaib</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1239,11 +1451,23 @@
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
         <v>0</v>
       </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1251,12 +1475,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Najam Bajwa</t>
+          <t>Najam Saqib</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Poppi</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1286,11 +1510,23 @@
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2025-02-01</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
         <v>0</v>
       </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1333,11 +1569,23 @@
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2025-07-20</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
         <v>0</v>
       </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: implement 6-month expiry for carried leaves and reset current balance
</commit_message>
<xml_diff>
--- a/Emp_data.xlsx
+++ b/Emp_data.xlsx
@@ -531,16 +531,16 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>11.5</v>
+        <v>14</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -564,7 +564,7 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -806,10 +806,8 @@
         <v>0</v>
       </c>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>03365111740</t>
-        </is>
+      <c r="S6" t="n">
+        <v>3365111740</v>
       </c>
     </row>
     <row r="7">
@@ -1046,10 +1044,8 @@
         <v>0</v>
       </c>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>03245494440</t>
-        </is>
+      <c r="S10" t="n">
+        <v>3245494440</v>
       </c>
     </row>
     <row r="11">
@@ -1168,10 +1164,8 @@
         <v>0</v>
       </c>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>03365404410</t>
-        </is>
+      <c r="S12" t="n">
+        <v>3365404410</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
feat: updated Hafiz Zohaib phone number and production logic
</commit_message>
<xml_diff>
--- a/Emp_data.xlsx
+++ b/Emp_data.xlsx
@@ -806,8 +806,10 @@
         <v>0</v>
       </c>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="n">
-        <v>3365111740</v>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>03365111740</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1044,8 +1046,10 @@
         <v>0</v>
       </c>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="n">
-        <v>3245494440</v>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>3245494440.0</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1164,8 +1168,10 @@
         <v>0</v>
       </c>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="n">
-        <v>3365404410</v>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>3365404410.0</t>
+        </is>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
feat: updated all employee names to use underscores instead of spaces
</commit_message>
<xml_diff>
--- a/Emp_data.xlsx
+++ b/Emp_data.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Muhammad Ahsan</t>
+          <t>Muhammad_Ahsan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ismail Anwar</t>
+          <t>Ismail_Anwar</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Haris Saeed</t>
+          <t>Haris_Saeed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abdul Hadi</t>
+          <t>Abdul_Hadi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hafiz Zohaib</t>
+          <t>Hafiz_Zohaib</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -806,10 +806,8 @@
         <v>0</v>
       </c>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>03365111740</t>
-        </is>
+      <c r="S6" t="n">
+        <v>3365111740</v>
       </c>
     </row>
     <row r="7">
@@ -818,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tanzeel Abid</t>
+          <t>Tanzeel_Abid</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -995,7 +993,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sajeel Fasihi</t>
+          <t>Sajeel_Fasihi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1046,10 +1044,8 @@
         <v>0</v>
       </c>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>3245494440.0</t>
-        </is>
+      <c r="S10" t="n">
+        <v>3245494440</v>
       </c>
     </row>
     <row r="11">
@@ -1058,7 +1054,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yasir Nawaz</t>
+          <t>Yasir_Nawaz</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1117,7 +1113,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hatif Javed</t>
+          <t>Hatif_Javed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1168,10 +1164,8 @@
         <v>0</v>
       </c>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>3365404410.0</t>
-        </is>
+      <c r="S12" t="n">
+        <v>3365404410</v>
       </c>
     </row>
     <row r="13">
@@ -1180,7 +1174,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Moeed Iftikhar</t>
+          <t>Moeed_Iftikhar</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1475,7 +1469,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Najam Saqib</t>
+          <t>Najam_Saqib</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">

</xml_diff>